<commit_message>
Fixed company_name && phone BUG
</commit_message>
<xml_diff>
--- a/excel_all.xlsx
+++ b/excel_all.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20386"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20390"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jackey\Desktop\github\work-order\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E9DFEE4-8B7A-4C3A-945D-1BBC16CACC23}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F734374-7218-4BED-A6C3-82C9B189AE77}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="10133" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -144,10 +144,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>特殊計價</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>稅額</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -157,6 +153,10 @@
   </si>
   <si>
     <t>總計</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>備料計價</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1281,7 +1281,7 @@
         <v>38</v>
       </c>
       <c r="N3" s="22" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="33" x14ac:dyDescent="1.05">
@@ -1540,7 +1540,7 @@
       <c r="I19" s="35"/>
       <c r="J19" s="23"/>
       <c r="K19" s="41" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L19" s="42"/>
       <c r="M19" s="3"/>
@@ -1594,7 +1594,7 @@
       <c r="I21" s="26"/>
       <c r="J21" s="23"/>
       <c r="K21" s="43" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L21" s="44"/>
       <c r="M21" s="3"/>
@@ -1646,7 +1646,7 @@
       <c r="I23" s="26"/>
       <c r="J23" s="23"/>
       <c r="K23" s="43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L23" s="44"/>
       <c r="M23" s="3"/>

</xml_diff>